<commit_message>
Add data cleaning stage and refresh source data
</commit_message>
<xml_diff>
--- a/Data/customer_churn_data_raw.xlsx
+++ b/Data/customer_churn_data_raw.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shail\Documents\SBundhun_Dev\Analytical_Dev\Customer_Churn_Analysis\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB21B3E0-9A3F-44CA-A323-A3F90F86967E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A355EA68-A0B4-45D7-B752-51EF4D5B9E19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AFD57064-DCB2-462B-A9F2-3B79D856F662}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="12150" windowHeight="20685" xr2:uid="{AFD57064-DCB2-462B-A9F2-3B79D856F662}"/>
   </bookViews>
   <sheets>
     <sheet name="db_customer" sheetId="1" r:id="rId1"/>
@@ -408,9 +408,6 @@
     <t>state</t>
   </si>
   <si>
-    <t>Toronto</t>
-  </si>
-  <si>
     <t>Canada</t>
   </si>
   <si>
@@ -493,6 +490,9 @@
   </si>
   <si>
     <t>pristina</t>
+  </si>
+  <si>
+    <t>Ontario</t>
   </si>
 </sst>
 </file>
@@ -1032,13 +1032,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>22</v>
@@ -1055,13 +1055,13 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>22</v>
@@ -1075,13 +1075,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>21</v>
@@ -1098,13 +1098,13 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>22</v>
@@ -1118,13 +1118,13 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>21</v>
@@ -1141,10 +1141,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>91</v>
@@ -1158,13 +1158,13 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C8" t="s">
+        <v>122</v>
+      </c>
+      <c r="D8" t="s">
         <v>123</v>
-      </c>
-      <c r="D8" t="s">
-        <v>124</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>21</v>
@@ -1178,13 +1178,13 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>22</v>
@@ -1201,7 +1201,7 @@
         <v>116</v>
       </c>
       <c r="D10" t="s">
-        <v>121</v>
+        <v>149</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>91</v>
@@ -1218,10 +1218,10 @@
         <v>115</v>
       </c>
       <c r="C11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D11" t="s">
-        <v>121</v>
+        <v>149</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>22</v>
@@ -1238,10 +1238,10 @@
         <v>114</v>
       </c>
       <c r="C12" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D12" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>92</v>
@@ -1255,13 +1255,13 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>21</v>
@@ -1275,10 +1275,10 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D14" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>21</v>
@@ -1292,13 +1292,13 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>21</v>
@@ -1312,13 +1312,13 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C16" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D16" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>92</v>
@@ -1332,13 +1332,13 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C17" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D17" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>21</v>
@@ -1355,13 +1355,13 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C18" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D18" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>21</v>
@@ -1375,13 +1375,13 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D19" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>21</v>
@@ -1395,13 +1395,13 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C20" t="s">
         <v>122</v>
       </c>
       <c r="D20" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>22</v>
@@ -1415,13 +1415,13 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C21" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D21" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>92</v>
@@ -1435,13 +1435,13 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C22" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D22" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>91</v>

</xml_diff>